<commit_message>
Volví a correr el assess_model para todos los países y cambie de modelo para ITA, GER y ARG.
</commit_message>
<xml_diff>
--- a/data/argentina/p6_deployment/missing/data_understanding/all/df_match_odds_miss.xlsx
+++ b/data/argentina/p6_deployment/missing/data_understanding/all/df_match_odds_miss.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D596"/>
+  <dimension ref="A1:D663"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9411,20 +9411,14 @@
           <t>SvlzcWFD</t>
         </is>
       </c>
-      <c r="B562" t="inlineStr">
-        <is>
-          <t>1.62</t>
-        </is>
-      </c>
-      <c r="C562" t="inlineStr">
-        <is>
-          <t>3.50</t>
-        </is>
-      </c>
-      <c r="D562" t="inlineStr">
-        <is>
-          <t>6.50</t>
-        </is>
+      <c r="B562" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="C562" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="D562" t="n">
+        <v>6.5</v>
       </c>
     </row>
     <row r="563">
@@ -9433,20 +9427,14 @@
           <t>65Xumenk</t>
         </is>
       </c>
-      <c r="B563" t="inlineStr">
-        <is>
-          <t>2.50</t>
-        </is>
-      </c>
-      <c r="C563" t="inlineStr">
-        <is>
-          <t>2.80</t>
-        </is>
-      </c>
-      <c r="D563" t="inlineStr">
-        <is>
-          <t>3.40</t>
-        </is>
+      <c r="B563" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C563" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="D563" t="n">
+        <v>3.4</v>
       </c>
     </row>
     <row r="564">
@@ -9455,20 +9443,14 @@
           <t>8fN0daP2</t>
         </is>
       </c>
-      <c r="B564" t="inlineStr">
-        <is>
-          <t>2.40</t>
-        </is>
-      </c>
-      <c r="C564" t="inlineStr">
-        <is>
-          <t>3.10</t>
-        </is>
-      </c>
-      <c r="D564" t="inlineStr">
-        <is>
-          <t>3.20</t>
-        </is>
+      <c r="B564" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="C564" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="D564" t="n">
+        <v>3.2</v>
       </c>
     </row>
     <row r="565">
@@ -9477,20 +9459,14 @@
           <t>jJjztvuM</t>
         </is>
       </c>
-      <c r="B565" t="inlineStr">
-        <is>
-          <t>2.63</t>
-        </is>
-      </c>
-      <c r="C565" t="inlineStr">
-        <is>
-          <t>2.90</t>
-        </is>
-      </c>
-      <c r="D565" t="inlineStr">
-        <is>
-          <t>3.00</t>
-        </is>
+      <c r="B565" t="n">
+        <v>2.63</v>
+      </c>
+      <c r="C565" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="D565" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="566">
@@ -9499,20 +9475,14 @@
           <t>rDFDgc9L</t>
         </is>
       </c>
-      <c r="B566" t="inlineStr">
-        <is>
-          <t>1.83</t>
-        </is>
-      </c>
-      <c r="C566" t="inlineStr">
-        <is>
-          <t>3.10</t>
-        </is>
-      </c>
-      <c r="D566" t="inlineStr">
-        <is>
-          <t>5.50</t>
-        </is>
+      <c r="B566" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="C566" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="D566" t="n">
+        <v>5.5</v>
       </c>
     </row>
     <row r="567">
@@ -9521,20 +9491,14 @@
           <t>U9kvubfS</t>
         </is>
       </c>
-      <c r="B567" t="inlineStr">
-        <is>
-          <t>1.80</t>
-        </is>
-      </c>
-      <c r="C567" t="inlineStr">
-        <is>
-          <t>3.60</t>
-        </is>
-      </c>
-      <c r="D567" t="inlineStr">
-        <is>
-          <t>4.50</t>
-        </is>
+      <c r="B567" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="C567" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="D567" t="n">
+        <v>4.5</v>
       </c>
     </row>
     <row r="568">
@@ -9543,20 +9507,14 @@
           <t>xzFHhHOR</t>
         </is>
       </c>
-      <c r="B568" t="inlineStr">
-        <is>
-          <t>1.53</t>
-        </is>
-      </c>
-      <c r="C568" t="inlineStr">
-        <is>
-          <t>3.90</t>
-        </is>
-      </c>
-      <c r="D568" t="inlineStr">
-        <is>
-          <t>7.00</t>
-        </is>
+      <c r="B568" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="C568" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="D568" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="569">
@@ -9565,20 +9523,14 @@
           <t>bPuAZyIk</t>
         </is>
       </c>
-      <c r="B569" t="inlineStr">
-        <is>
-          <t>2.75</t>
-        </is>
-      </c>
-      <c r="C569" t="inlineStr">
-        <is>
-          <t>2.75</t>
-        </is>
-      </c>
-      <c r="D569" t="inlineStr">
-        <is>
-          <t>3.00</t>
-        </is>
+      <c r="B569" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C569" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="D569" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="570">
@@ -9587,20 +9539,14 @@
           <t>tlVEYeXe</t>
         </is>
       </c>
-      <c r="B570" t="inlineStr">
-        <is>
-          <t>3.50</t>
-        </is>
-      </c>
-      <c r="C570" t="inlineStr">
-        <is>
-          <t>3.10</t>
-        </is>
-      </c>
-      <c r="D570" t="inlineStr">
-        <is>
-          <t>2.20</t>
-        </is>
+      <c r="B570" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="C570" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="D570" t="n">
+        <v>2.2</v>
       </c>
     </row>
     <row r="571">
@@ -9609,20 +9555,14 @@
           <t>KvUIXFn2</t>
         </is>
       </c>
-      <c r="B571" t="inlineStr">
-        <is>
-          <t>3.80</t>
-        </is>
-      </c>
-      <c r="C571" t="inlineStr">
-        <is>
-          <t>3.25</t>
-        </is>
-      </c>
-      <c r="D571" t="inlineStr">
-        <is>
-          <t>2.05</t>
-        </is>
+      <c r="B571" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="C571" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="D571" t="n">
+        <v>2.05</v>
       </c>
     </row>
     <row r="572">
@@ -9631,20 +9571,14 @@
           <t>U9B9fwfF</t>
         </is>
       </c>
-      <c r="B572" t="inlineStr">
-        <is>
-          <t>1.85</t>
-        </is>
-      </c>
-      <c r="C572" t="inlineStr">
-        <is>
-          <t>3.20</t>
-        </is>
-      </c>
-      <c r="D572" t="inlineStr">
-        <is>
-          <t>5.25</t>
-        </is>
+      <c r="B572" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="C572" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="D572" t="n">
+        <v>5.25</v>
       </c>
     </row>
     <row r="573">
@@ -9653,20 +9587,14 @@
           <t>vq1qlyXr</t>
         </is>
       </c>
-      <c r="B573" t="inlineStr">
-        <is>
-          <t>2.15</t>
-        </is>
-      </c>
-      <c r="C573" t="inlineStr">
-        <is>
-          <t>3.10</t>
-        </is>
-      </c>
-      <c r="D573" t="inlineStr">
-        <is>
-          <t>3.70</t>
-        </is>
+      <c r="B573" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="C573" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="D573" t="n">
+        <v>3.7</v>
       </c>
     </row>
     <row r="574">
@@ -9675,20 +9603,14 @@
           <t>nkx6zI2q</t>
         </is>
       </c>
-      <c r="B574" t="inlineStr">
-        <is>
-          <t>1.75</t>
-        </is>
-      </c>
-      <c r="C574" t="inlineStr">
-        <is>
-          <t>3.30</t>
-        </is>
-      </c>
-      <c r="D574" t="inlineStr">
-        <is>
-          <t>5.25</t>
-        </is>
+      <c r="B574" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="C574" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="D574" t="n">
+        <v>5.25</v>
       </c>
     </row>
     <row r="575">
@@ -9697,20 +9619,14 @@
           <t>pdWqnF1e</t>
         </is>
       </c>
-      <c r="B575" t="inlineStr">
-        <is>
-          <t>1.85</t>
-        </is>
-      </c>
-      <c r="C575" t="inlineStr">
-        <is>
-          <t>3.40</t>
-        </is>
-      </c>
-      <c r="D575" t="inlineStr">
-        <is>
-          <t>4.33</t>
-        </is>
+      <c r="B575" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="C575" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="D575" t="n">
+        <v>4.33</v>
       </c>
     </row>
     <row r="576">
@@ -9719,20 +9635,14 @@
           <t>noM4eJv9</t>
         </is>
       </c>
-      <c r="B576" t="inlineStr">
-        <is>
-          <t>3.00</t>
-        </is>
-      </c>
-      <c r="C576" t="inlineStr">
-        <is>
-          <t>2.88</t>
-        </is>
-      </c>
-      <c r="D576" t="inlineStr">
-        <is>
-          <t>2.75</t>
-        </is>
+      <c r="B576" t="n">
+        <v>3</v>
+      </c>
+      <c r="C576" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="D576" t="n">
+        <v>2.75</v>
       </c>
     </row>
     <row r="577">
@@ -9741,20 +9651,14 @@
           <t>xCbnCYTO</t>
         </is>
       </c>
-      <c r="B577" t="inlineStr">
-        <is>
-          <t>1.62</t>
-        </is>
-      </c>
-      <c r="C577" t="inlineStr">
-        <is>
-          <t>3.30</t>
-        </is>
-      </c>
-      <c r="D577" t="inlineStr">
-        <is>
-          <t>6.50</t>
-        </is>
+      <c r="B577" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="C577" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="D577" t="n">
+        <v>6.5</v>
       </c>
     </row>
     <row r="578">
@@ -9763,20 +9667,14 @@
           <t>4M6ZEzp6</t>
         </is>
       </c>
-      <c r="B578" t="inlineStr">
-        <is>
-          <t>2.55</t>
-        </is>
-      </c>
-      <c r="C578" t="inlineStr">
-        <is>
-          <t>2.80</t>
-        </is>
-      </c>
-      <c r="D578" t="inlineStr">
-        <is>
-          <t>3.10</t>
-        </is>
+      <c r="B578" t="n">
+        <v>2.55</v>
+      </c>
+      <c r="C578" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="D578" t="n">
+        <v>3.1</v>
       </c>
     </row>
     <row r="579">
@@ -9785,20 +9683,14 @@
           <t>IPW8TZba</t>
         </is>
       </c>
-      <c r="B579" t="inlineStr">
-        <is>
-          <t>2.75</t>
-        </is>
-      </c>
-      <c r="C579" t="inlineStr">
-        <is>
-          <t>2.80</t>
-        </is>
-      </c>
-      <c r="D579" t="inlineStr">
-        <is>
-          <t>3.00</t>
-        </is>
+      <c r="B579" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C579" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="D579" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="580">
@@ -9807,20 +9699,14 @@
           <t>bLarDEEI</t>
         </is>
       </c>
-      <c r="B580" t="inlineStr">
-        <is>
-          <t>2.50</t>
-        </is>
-      </c>
-      <c r="C580" t="inlineStr">
-        <is>
-          <t>2.88</t>
-        </is>
-      </c>
-      <c r="D580" t="inlineStr">
-        <is>
-          <t>3.20</t>
-        </is>
+      <c r="B580" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C580" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="D580" t="n">
+        <v>3.2</v>
       </c>
     </row>
     <row r="581">
@@ -9829,20 +9715,14 @@
           <t>SzvdWyFt</t>
         </is>
       </c>
-      <c r="B581" t="inlineStr">
-        <is>
-          <t>2.88</t>
-        </is>
-      </c>
-      <c r="C581" t="inlineStr">
-        <is>
-          <t>2.75</t>
-        </is>
-      </c>
-      <c r="D581" t="inlineStr">
-        <is>
-          <t>2.88</t>
-        </is>
+      <c r="B581" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="C581" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="D581" t="n">
+        <v>2.88</v>
       </c>
     </row>
     <row r="582">
@@ -9851,20 +9731,14 @@
           <t>W88RGdFg</t>
         </is>
       </c>
-      <c r="B582" t="inlineStr">
-        <is>
-          <t>2.20</t>
-        </is>
-      </c>
-      <c r="C582" t="inlineStr">
-        <is>
-          <t>3.10</t>
-        </is>
-      </c>
-      <c r="D582" t="inlineStr">
-        <is>
-          <t>3.60</t>
-        </is>
+      <c r="B582" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="C582" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="D582" t="n">
+        <v>3.6</v>
       </c>
     </row>
     <row r="583">
@@ -9873,20 +9747,14 @@
           <t>GIoEQXrI</t>
         </is>
       </c>
-      <c r="B583" t="inlineStr">
-        <is>
-          <t>2.10</t>
-        </is>
-      </c>
-      <c r="C583" t="inlineStr">
-        <is>
-          <t>3.00</t>
-        </is>
-      </c>
-      <c r="D583" t="inlineStr">
-        <is>
-          <t>4.00</t>
-        </is>
+      <c r="B583" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="C583" t="n">
+        <v>3</v>
+      </c>
+      <c r="D583" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="584">
@@ -9895,20 +9763,14 @@
           <t>4bOnOvNJ</t>
         </is>
       </c>
-      <c r="B584" t="inlineStr">
-        <is>
-          <t>2.35</t>
-        </is>
-      </c>
-      <c r="C584" t="inlineStr">
-        <is>
-          <t>2.88</t>
-        </is>
-      </c>
-      <c r="D584" t="inlineStr">
-        <is>
-          <t>3.50</t>
-        </is>
+      <c r="B584" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="C584" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="D584" t="n">
+        <v>3.5</v>
       </c>
     </row>
     <row r="585">
@@ -9917,20 +9779,14 @@
           <t>zsFIIIps</t>
         </is>
       </c>
-      <c r="B585" t="inlineStr">
-        <is>
-          <t>1.90</t>
-        </is>
-      </c>
-      <c r="C585" t="inlineStr">
-        <is>
-          <t>3.30</t>
-        </is>
-      </c>
-      <c r="D585" t="inlineStr">
-        <is>
-          <t>4.20</t>
-        </is>
+      <c r="B585" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="C585" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="D585" t="n">
+        <v>4.2</v>
       </c>
     </row>
     <row r="586">
@@ -9939,20 +9795,14 @@
           <t>EXDMHx0m</t>
         </is>
       </c>
-      <c r="B586" t="inlineStr">
-        <is>
-          <t>2.10</t>
-        </is>
-      </c>
-      <c r="C586" t="inlineStr">
-        <is>
-          <t>2.75</t>
-        </is>
-      </c>
-      <c r="D586" t="inlineStr">
-        <is>
-          <t>4.33</t>
-        </is>
+      <c r="B586" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="C586" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="D586" t="n">
+        <v>4.33</v>
       </c>
     </row>
     <row r="587">
@@ -9961,20 +9811,14 @@
           <t>dGVCSgE5</t>
         </is>
       </c>
-      <c r="B587" t="inlineStr">
-        <is>
-          <t>1.67</t>
-        </is>
-      </c>
-      <c r="C587" t="inlineStr">
-        <is>
-          <t>3.40</t>
-        </is>
-      </c>
-      <c r="D587" t="inlineStr">
-        <is>
-          <t>5.50</t>
-        </is>
+      <c r="B587" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="C587" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="D587" t="n">
+        <v>5.5</v>
       </c>
     </row>
     <row r="588">
@@ -9983,20 +9827,14 @@
           <t>GdAwEfaC</t>
         </is>
       </c>
-      <c r="B588" t="inlineStr">
-        <is>
-          <t>2.10</t>
-        </is>
-      </c>
-      <c r="C588" t="inlineStr">
-        <is>
-          <t>2.90</t>
-        </is>
-      </c>
-      <c r="D588" t="inlineStr">
-        <is>
-          <t>4.00</t>
-        </is>
+      <c r="B588" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="C588" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="D588" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="589">
@@ -10005,20 +9843,14 @@
           <t>QRiUzI6P</t>
         </is>
       </c>
-      <c r="B589" t="inlineStr">
-        <is>
-          <t>2.25</t>
-        </is>
-      </c>
-      <c r="C589" t="inlineStr">
-        <is>
-          <t>2.80</t>
-        </is>
-      </c>
-      <c r="D589" t="inlineStr">
-        <is>
-          <t>3.75</t>
-        </is>
+      <c r="B589" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="C589" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="D589" t="n">
+        <v>3.75</v>
       </c>
     </row>
     <row r="590">
@@ -10027,20 +9859,14 @@
           <t>xSnARDTB</t>
         </is>
       </c>
-      <c r="B590" t="inlineStr">
-        <is>
-          <t>1.90</t>
-        </is>
-      </c>
-      <c r="C590" t="inlineStr">
-        <is>
-          <t>2.90</t>
-        </is>
-      </c>
-      <c r="D590" t="inlineStr">
-        <is>
-          <t>5.00</t>
-        </is>
+      <c r="B590" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="C590" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="D590" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="591">
@@ -10049,20 +9875,14 @@
           <t>AaT0VeUn</t>
         </is>
       </c>
-      <c r="B591" t="inlineStr">
-        <is>
-          <t>3.10</t>
-        </is>
-      </c>
-      <c r="C591" t="inlineStr">
-        <is>
-          <t>2.70</t>
-        </is>
-      </c>
-      <c r="D591" t="inlineStr">
-        <is>
-          <t>2.63</t>
-        </is>
+      <c r="B591" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="C591" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="D591" t="n">
+        <v>2.63</v>
       </c>
     </row>
     <row r="592">
@@ -10071,20 +9891,14 @@
           <t>O2X4UFqg</t>
         </is>
       </c>
-      <c r="B592" t="inlineStr">
-        <is>
-          <t>1.62</t>
-        </is>
-      </c>
-      <c r="C592" t="inlineStr">
-        <is>
-          <t>3.30</t>
-        </is>
-      </c>
-      <c r="D592" t="inlineStr">
-        <is>
-          <t>7.50</t>
-        </is>
+      <c r="B592" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="C592" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="D592" t="n">
+        <v>7.5</v>
       </c>
     </row>
     <row r="593">
@@ -10093,20 +9907,14 @@
           <t>2gp4aepJ</t>
         </is>
       </c>
-      <c r="B593" t="inlineStr">
-        <is>
-          <t>2.50</t>
-        </is>
-      </c>
-      <c r="C593" t="inlineStr">
-        <is>
-          <t>2.63</t>
-        </is>
-      </c>
-      <c r="D593" t="inlineStr">
-        <is>
-          <t>3.50</t>
-        </is>
+      <c r="B593" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C593" t="n">
+        <v>2.63</v>
+      </c>
+      <c r="D593" t="n">
+        <v>3.5</v>
       </c>
     </row>
     <row r="594">
@@ -10115,20 +9923,14 @@
           <t>I1SjNbxQ</t>
         </is>
       </c>
-      <c r="B594" t="inlineStr">
-        <is>
-          <t>2.00</t>
-        </is>
-      </c>
-      <c r="C594" t="inlineStr">
-        <is>
-          <t>2.88</t>
-        </is>
-      </c>
-      <c r="D594" t="inlineStr">
-        <is>
-          <t>5.00</t>
-        </is>
+      <c r="B594" t="n">
+        <v>2</v>
+      </c>
+      <c r="C594" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="D594" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="595">
@@ -10137,20 +9939,14 @@
           <t>Aa7VFGUa</t>
         </is>
       </c>
-      <c r="B595" t="inlineStr">
-        <is>
-          <t>1.67</t>
-        </is>
-      </c>
-      <c r="C595" t="inlineStr">
-        <is>
-          <t>3.40</t>
-        </is>
-      </c>
-      <c r="D595" t="inlineStr">
-        <is>
-          <t>5.25</t>
-        </is>
+      <c r="B595" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="C595" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="D595" t="n">
+        <v>5.25</v>
       </c>
     </row>
     <row r="596">
@@ -10159,19 +9955,1487 @@
           <t>ngdGLTFj</t>
         </is>
       </c>
-      <c r="B596" t="inlineStr">
-        <is>
-          <t>3.45</t>
-        </is>
-      </c>
-      <c r="C596" t="inlineStr">
-        <is>
-          <t>2.65</t>
-        </is>
-      </c>
-      <c r="D596" t="inlineStr">
-        <is>
-          <t>2.48</t>
+      <c r="B596" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="C596" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="D596" t="n">
+        <v>2.48</v>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" s="1" t="inlineStr">
+        <is>
+          <t>On7sciXA</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>2.35</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>3.20</t>
+        </is>
+      </c>
+      <c r="D597" t="inlineStr">
+        <is>
+          <t>3.25</t>
+        </is>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" s="1" t="inlineStr">
+        <is>
+          <t>vJHhFDVs</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>1.65</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>3.40</t>
+        </is>
+      </c>
+      <c r="D598" t="inlineStr">
+        <is>
+          <t>6.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" s="1" t="inlineStr">
+        <is>
+          <t>QZF0Di0f</t>
+        </is>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>2.25</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>2.80</t>
+        </is>
+      </c>
+      <c r="D599" t="inlineStr">
+        <is>
+          <t>4.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" s="1" t="inlineStr">
+        <is>
+          <t>8b55CBF0</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>1.48</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>4.00</t>
+        </is>
+      </c>
+      <c r="D600" t="inlineStr">
+        <is>
+          <t>7.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" s="1" t="inlineStr">
+        <is>
+          <t>WY1N1FIu</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>2.45</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>2.90</t>
+        </is>
+      </c>
+      <c r="D601" t="inlineStr">
+        <is>
+          <t>3.40</t>
+        </is>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" s="1" t="inlineStr">
+        <is>
+          <t>nqHdEXpl</t>
+        </is>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>2.80</t>
+        </is>
+      </c>
+      <c r="C602" t="inlineStr">
+        <is>
+          <t>2.88</t>
+        </is>
+      </c>
+      <c r="D602" t="inlineStr">
+        <is>
+          <t>2.88</t>
+        </is>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" s="1" t="inlineStr">
+        <is>
+          <t>AP0R0ZXo</t>
+        </is>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>1.80</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>3.30</t>
+        </is>
+      </c>
+      <c r="D603" t="inlineStr">
+        <is>
+          <t>5.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" s="1" t="inlineStr">
+        <is>
+          <t>4n0Vagmh</t>
+        </is>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>2.05</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>3.25</t>
+        </is>
+      </c>
+      <c r="D604" t="inlineStr">
+        <is>
+          <t>3.90</t>
+        </is>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" s="1" t="inlineStr">
+        <is>
+          <t>pd8wbXH4</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>2.00</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>3.20</t>
+        </is>
+      </c>
+      <c r="D605" t="inlineStr">
+        <is>
+          <t>4.20</t>
+        </is>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" s="1" t="inlineStr">
+        <is>
+          <t>M199BVU6</t>
+        </is>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>3.50</t>
+        </is>
+      </c>
+      <c r="C606" t="inlineStr">
+        <is>
+          <t>3.20</t>
+        </is>
+      </c>
+      <c r="D606" t="inlineStr">
+        <is>
+          <t>2.20</t>
+        </is>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" s="1" t="inlineStr">
+        <is>
+          <t>fF7H99aJ</t>
+        </is>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>1.65</t>
+        </is>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>3.10</t>
+        </is>
+      </c>
+      <c r="D607" t="inlineStr">
+        <is>
+          <t>8.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" s="1" t="inlineStr">
+        <is>
+          <t>xAVQJgNQ</t>
+        </is>
+      </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>2.10</t>
+        </is>
+      </c>
+      <c r="C608" t="inlineStr">
+        <is>
+          <t>3.00</t>
+        </is>
+      </c>
+      <c r="D608" t="inlineStr">
+        <is>
+          <t>4.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" s="1" t="inlineStr">
+        <is>
+          <t>GO8DAkpD</t>
+        </is>
+      </c>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>3.30</t>
+        </is>
+      </c>
+      <c r="C609" t="inlineStr">
+        <is>
+          <t>3.10</t>
+        </is>
+      </c>
+      <c r="D609" t="inlineStr">
+        <is>
+          <t>2.38</t>
+        </is>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" s="1" t="inlineStr">
+        <is>
+          <t>2XIYbD2b</t>
+        </is>
+      </c>
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>1.73</t>
+        </is>
+      </c>
+      <c r="C610" t="inlineStr">
+        <is>
+          <t>3.20</t>
+        </is>
+      </c>
+      <c r="D610" t="inlineStr">
+        <is>
+          <t>6.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" s="1" t="inlineStr">
+        <is>
+          <t>trxILFhE</t>
+        </is>
+      </c>
+      <c r="B611" t="inlineStr">
+        <is>
+          <t>2.35</t>
+        </is>
+      </c>
+      <c r="C611" t="inlineStr">
+        <is>
+          <t>3.00</t>
+        </is>
+      </c>
+      <c r="D611" t="inlineStr">
+        <is>
+          <t>3.40</t>
+        </is>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" s="1" t="inlineStr">
+        <is>
+          <t>nPhF1f1r</t>
+        </is>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>2.05</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>2.80</t>
+        </is>
+      </c>
+      <c r="D612" t="inlineStr">
+        <is>
+          <t>4.75</t>
+        </is>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" s="1" t="inlineStr">
+        <is>
+          <t>hMZipgW7</t>
+        </is>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>3.60</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>3.00</t>
+        </is>
+      </c>
+      <c r="D613" t="inlineStr">
+        <is>
+          <t>2.25</t>
+        </is>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" s="1" t="inlineStr">
+        <is>
+          <t>vJVmoZG1</t>
+        </is>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>2.63</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr">
+        <is>
+          <t>3.10</t>
+        </is>
+      </c>
+      <c r="D614" t="inlineStr">
+        <is>
+          <t>2.80</t>
+        </is>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" s="1" t="inlineStr">
+        <is>
+          <t>fRDz9x98</t>
+        </is>
+      </c>
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>1.85</t>
+        </is>
+      </c>
+      <c r="C615" t="inlineStr">
+        <is>
+          <t>3.20</t>
+        </is>
+      </c>
+      <c r="D615" t="inlineStr">
+        <is>
+          <t>5.25</t>
+        </is>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" s="1" t="inlineStr">
+        <is>
+          <t>WCfRbho1</t>
+        </is>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>1.67</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>3.60</t>
+        </is>
+      </c>
+      <c r="D616" t="inlineStr">
+        <is>
+          <t>5.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" s="1" t="inlineStr">
+        <is>
+          <t>2iHr7GwL</t>
+        </is>
+      </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>3.70</t>
+        </is>
+      </c>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>2.90</t>
+        </is>
+      </c>
+      <c r="D617" t="inlineStr">
+        <is>
+          <t>2.30</t>
+        </is>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" s="1" t="inlineStr">
+        <is>
+          <t>badJ0EGl</t>
+        </is>
+      </c>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>2.30</t>
+        </is>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>2.70</t>
+        </is>
+      </c>
+      <c r="D618" t="inlineStr">
+        <is>
+          <t>3.80</t>
+        </is>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" s="1" t="inlineStr">
+        <is>
+          <t>trGn6zgR</t>
+        </is>
+      </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>2.35</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr">
+        <is>
+          <t>2.75</t>
+        </is>
+      </c>
+      <c r="D619" t="inlineStr">
+        <is>
+          <t>3.80</t>
+        </is>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" s="1" t="inlineStr">
+        <is>
+          <t>hMeNaYVf</t>
+        </is>
+      </c>
+      <c r="B620" t="inlineStr">
+        <is>
+          <t>1.67</t>
+        </is>
+      </c>
+      <c r="C620" t="inlineStr">
+        <is>
+          <t>3.70</t>
+        </is>
+      </c>
+      <c r="D620" t="inlineStr">
+        <is>
+          <t>5.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" s="1" t="inlineStr">
+        <is>
+          <t>llkWcC07</t>
+        </is>
+      </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>2.55</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>2.75</t>
+        </is>
+      </c>
+      <c r="D621" t="inlineStr">
+        <is>
+          <t>3.40</t>
+        </is>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" s="1" t="inlineStr">
+        <is>
+          <t>YHCv8dOE</t>
+        </is>
+      </c>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>3.75</t>
+        </is>
+      </c>
+      <c r="C622" t="inlineStr">
+        <is>
+          <t>3.30</t>
+        </is>
+      </c>
+      <c r="D622" t="inlineStr">
+        <is>
+          <t>2.05</t>
+        </is>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" s="1" t="inlineStr">
+        <is>
+          <t>fotMKZ7K</t>
+        </is>
+      </c>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>3.70</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr">
+        <is>
+          <t>3.10</t>
+        </is>
+      </c>
+      <c r="D623" t="inlineStr">
+        <is>
+          <t>2.15</t>
+        </is>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" s="1" t="inlineStr">
+        <is>
+          <t>KtcNbhUl</t>
+        </is>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>2.00</t>
+        </is>
+      </c>
+      <c r="C624" t="inlineStr">
+        <is>
+          <t>3.00</t>
+        </is>
+      </c>
+      <c r="D624" t="inlineStr">
+        <is>
+          <t>4.20</t>
+        </is>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" s="1" t="inlineStr">
+        <is>
+          <t>YFg0qDU1</t>
+        </is>
+      </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>2.15</t>
+        </is>
+      </c>
+      <c r="C625" t="inlineStr">
+        <is>
+          <t>3.00</t>
+        </is>
+      </c>
+      <c r="D625" t="inlineStr">
+        <is>
+          <t>3.90</t>
+        </is>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" s="1" t="inlineStr">
+        <is>
+          <t>KIEz8d72</t>
+        </is>
+      </c>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>1.83</t>
+        </is>
+      </c>
+      <c r="C626" t="inlineStr">
+        <is>
+          <t>3.00</t>
+        </is>
+      </c>
+      <c r="D626" t="inlineStr">
+        <is>
+          <t>5.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" s="1" t="inlineStr">
+        <is>
+          <t>lb6i4E6R</t>
+        </is>
+      </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>2.05</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr">
+        <is>
+          <t>3.00</t>
+        </is>
+      </c>
+      <c r="D627" t="inlineStr">
+        <is>
+          <t>4.20</t>
+        </is>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" s="1" t="inlineStr">
+        <is>
+          <t>hWlzdjE7</t>
+        </is>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>2.00</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr">
+        <is>
+          <t>3.00</t>
+        </is>
+      </c>
+      <c r="D628" t="inlineStr">
+        <is>
+          <t>4.33</t>
+        </is>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" s="1" t="inlineStr">
+        <is>
+          <t>j7hJaYEr</t>
+        </is>
+      </c>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>2.88</t>
+        </is>
+      </c>
+      <c r="C629" t="inlineStr">
+        <is>
+          <t>2.75</t>
+        </is>
+      </c>
+      <c r="D629" t="inlineStr">
+        <is>
+          <t>2.88</t>
+        </is>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" s="1" t="inlineStr">
+        <is>
+          <t>6ZGn5fiL</t>
+        </is>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>1.80</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr">
+        <is>
+          <t>3.00</t>
+        </is>
+      </c>
+      <c r="D630" t="inlineStr">
+        <is>
+          <t>5.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" s="1" t="inlineStr">
+        <is>
+          <t>61wK3sGG</t>
+        </is>
+      </c>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>1.95</t>
+        </is>
+      </c>
+      <c r="C631" t="inlineStr">
+        <is>
+          <t>3.10</t>
+        </is>
+      </c>
+      <c r="D631" t="inlineStr">
+        <is>
+          <t>4.20</t>
+        </is>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" s="1" t="inlineStr">
+        <is>
+          <t>nailnFpq</t>
+        </is>
+      </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>1.90</t>
+        </is>
+      </c>
+      <c r="C632" t="inlineStr">
+        <is>
+          <t>3.30</t>
+        </is>
+      </c>
+      <c r="D632" t="inlineStr">
+        <is>
+          <t>4.20</t>
+        </is>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" s="1" t="inlineStr">
+        <is>
+          <t>hWCr6zxF</t>
+        </is>
+      </c>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>2.30</t>
+        </is>
+      </c>
+      <c r="C633" t="inlineStr">
+        <is>
+          <t>2.90</t>
+        </is>
+      </c>
+      <c r="D633" t="inlineStr">
+        <is>
+          <t>3.40</t>
+        </is>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" s="1" t="inlineStr">
+        <is>
+          <t>byzC53o4</t>
+        </is>
+      </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>1.91</t>
+        </is>
+      </c>
+      <c r="C634" t="inlineStr">
+        <is>
+          <t>3.10</t>
+        </is>
+      </c>
+      <c r="D634" t="inlineStr">
+        <is>
+          <t>4.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" s="1" t="inlineStr">
+        <is>
+          <t>bXeRcCqe</t>
+        </is>
+      </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>3.20</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>2.63</t>
+        </is>
+      </c>
+      <c r="D635" t="inlineStr">
+        <is>
+          <t>2.75</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" s="1" t="inlineStr">
+        <is>
+          <t>6ZxIKZj8</t>
+        </is>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>2.30</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>2.80</t>
+        </is>
+      </c>
+      <c r="D636" t="inlineStr">
+        <is>
+          <t>3.70</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" s="1" t="inlineStr">
+        <is>
+          <t>pQyMJg6E</t>
+        </is>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>3.00</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>2.75</t>
+        </is>
+      </c>
+      <c r="D637" t="inlineStr">
+        <is>
+          <t>2.75</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" s="1" t="inlineStr">
+        <is>
+          <t>SAvG4N0A</t>
+        </is>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>1.80</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>3.25</t>
+        </is>
+      </c>
+      <c r="D638" t="inlineStr">
+        <is>
+          <t>5.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" s="1" t="inlineStr">
+        <is>
+          <t>02ehoZak</t>
+        </is>
+      </c>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>2.15</t>
+        </is>
+      </c>
+      <c r="C639" t="inlineStr">
+        <is>
+          <t>3.00</t>
+        </is>
+      </c>
+      <c r="D639" t="inlineStr">
+        <is>
+          <t>3.70</t>
+        </is>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" s="1" t="inlineStr">
+        <is>
+          <t>fPfdpgFe</t>
+        </is>
+      </c>
+      <c r="B640" t="inlineStr">
+        <is>
+          <t>1.95</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr">
+        <is>
+          <t>3.00</t>
+        </is>
+      </c>
+      <c r="D640" t="inlineStr">
+        <is>
+          <t>4.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" s="1" t="inlineStr">
+        <is>
+          <t>b9Dv7GM8</t>
+        </is>
+      </c>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>2.70</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr">
+        <is>
+          <t>2.70</t>
+        </is>
+      </c>
+      <c r="D641" t="inlineStr">
+        <is>
+          <t>3.10</t>
+        </is>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" s="1" t="inlineStr">
+        <is>
+          <t>tdoWdWb1</t>
+        </is>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>1.62</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>3.40</t>
+        </is>
+      </c>
+      <c r="D642" t="inlineStr">
+        <is>
+          <t>6.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" s="1" t="inlineStr">
+        <is>
+          <t>E7EtjOoH</t>
+        </is>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>2.40</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>2.70</t>
+        </is>
+      </c>
+      <c r="D643" t="inlineStr">
+        <is>
+          <t>3.60</t>
+        </is>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" s="1" t="inlineStr">
+        <is>
+          <t>Qora851o</t>
+        </is>
+      </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>4.10</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>2.70</t>
+        </is>
+      </c>
+      <c r="D644" t="inlineStr">
+        <is>
+          <t>2.25</t>
+        </is>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" s="1" t="inlineStr">
+        <is>
+          <t>bBOHeSHu</t>
+        </is>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>3.00</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>2.75</t>
+        </is>
+      </c>
+      <c r="D645" t="inlineStr">
+        <is>
+          <t>2.75</t>
+        </is>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" s="1" t="inlineStr">
+        <is>
+          <t>lxFheb6a</t>
+        </is>
+      </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>2.50</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>2.63</t>
+        </is>
+      </c>
+      <c r="D646" t="inlineStr">
+        <is>
+          <t>3.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" s="1" t="inlineStr">
+        <is>
+          <t>SSDdfIL5</t>
+        </is>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>1.75</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>3.40</t>
+        </is>
+      </c>
+      <c r="D647" t="inlineStr">
+        <is>
+          <t>5.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" s="1" t="inlineStr">
+        <is>
+          <t>WKADjzLU</t>
+        </is>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>2.35</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>2.88</t>
+        </is>
+      </c>
+      <c r="D648" t="inlineStr">
+        <is>
+          <t>3.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" s="1" t="inlineStr">
+        <is>
+          <t>xMo37PGi</t>
+        </is>
+      </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>2.20</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>2.80</t>
+        </is>
+      </c>
+      <c r="D649" t="inlineStr">
+        <is>
+          <t>3.80</t>
+        </is>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" s="1" t="inlineStr">
+        <is>
+          <t>pSMPg6nh</t>
+        </is>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>2.40</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>2.90</t>
+        </is>
+      </c>
+      <c r="D650" t="inlineStr">
+        <is>
+          <t>3.25</t>
+        </is>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" s="1" t="inlineStr">
+        <is>
+          <t>6sBYipH4</t>
+        </is>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>3.30</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>2.63</t>
+        </is>
+      </c>
+      <c r="D651" t="inlineStr">
+        <is>
+          <t>2.63</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" s="1" t="inlineStr">
+        <is>
+          <t>Kpy86qWc</t>
+        </is>
+      </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>3.30</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>2.75</t>
+        </is>
+      </c>
+      <c r="D652" t="inlineStr">
+        <is>
+          <t>2.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" s="1" t="inlineStr">
+        <is>
+          <t>KpFxi4WA</t>
+        </is>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>2.70</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>2.63</t>
+        </is>
+      </c>
+      <c r="D653" t="inlineStr">
+        <is>
+          <t>3.25</t>
+        </is>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" s="1" t="inlineStr">
+        <is>
+          <t>OILThQ1b</t>
+        </is>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>1.95</t>
+        </is>
+      </c>
+      <c r="C654" t="inlineStr">
+        <is>
+          <t>3.00</t>
+        </is>
+      </c>
+      <c r="D654" t="inlineStr">
+        <is>
+          <t>4.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" s="1" t="inlineStr">
+        <is>
+          <t>CrfHqMOp</t>
+        </is>
+      </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>1.60</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr">
+        <is>
+          <t>3.60</t>
+        </is>
+      </c>
+      <c r="D655" t="inlineStr">
+        <is>
+          <t>6.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" s="1" t="inlineStr">
+        <is>
+          <t>IH69iG5O</t>
+        </is>
+      </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>2.75</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr">
+        <is>
+          <t>2.75</t>
+        </is>
+      </c>
+      <c r="D656" t="inlineStr">
+        <is>
+          <t>3.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" s="1" t="inlineStr">
+        <is>
+          <t>AZ7kl2GT</t>
+        </is>
+      </c>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>2.00</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>3.10</t>
+        </is>
+      </c>
+      <c r="D657" t="inlineStr">
+        <is>
+          <t>4.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" s="1" t="inlineStr">
+        <is>
+          <t>x2NLfnXo</t>
+        </is>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>1.95</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>3.00</t>
+        </is>
+      </c>
+      <c r="D658" t="inlineStr">
+        <is>
+          <t>4.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" s="1" t="inlineStr">
+        <is>
+          <t>Of75hdjI</t>
+        </is>
+      </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>1.67</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>3.30</t>
+        </is>
+      </c>
+      <c r="D659" t="inlineStr">
+        <is>
+          <t>6.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" s="1" t="inlineStr">
+        <is>
+          <t>p481gxyC</t>
+        </is>
+      </c>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>3.50</t>
+        </is>
+      </c>
+      <c r="C660" t="inlineStr">
+        <is>
+          <t>2.70</t>
+        </is>
+      </c>
+      <c r="D660" t="inlineStr">
+        <is>
+          <t>2.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" s="1" t="inlineStr">
+        <is>
+          <t>hbDpkr1N</t>
+        </is>
+      </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>2.00</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>3.10</t>
+        </is>
+      </c>
+      <c r="D661" t="inlineStr">
+        <is>
+          <t>4.20</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" s="1" t="inlineStr">
+        <is>
+          <t>fgvPVMI8</t>
+        </is>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>4.60</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>3.10</t>
+        </is>
+      </c>
+      <c r="D662" t="inlineStr">
+        <is>
+          <t>1.85</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" s="1" t="inlineStr">
+        <is>
+          <t>Y9EiyTMr</t>
+        </is>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>2.95</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>2.70</t>
+        </is>
+      </c>
+      <c r="D663" t="inlineStr">
+        <is>
+          <t>2.80</t>
         </is>
       </c>
     </row>

</xml_diff>